<commit_message>
Close the 8 unsourced lethal-risk cards with verified literature
Mexican GPC sites (.gob.mx), who.int and fda.gov are unreachable from the
build environment, so the missing sources come from PubMed/Consensus:
Cochrane (MgSO4 vs diazepam), CNGOF 2019 (no tocolysis with intrauterine
infection), Lee 2020 (tocolytics and atony), GASTRO 2019 and GASTROSAM
2025 (IV boluses for shock), Gilbertson 2019 and Spicer 1982 (pyloric
stenosis is a medical emergency first; the cited "AAP Clinical Report"
does not exist), Mann 2005 and Zalsman 2016 (means restriction), and the
2025 global Delphi consensus on clozapine (ANC monitoring for 2 years,
now stated in the mentor comment). Lethal-risk sheet: 45 approve, 18
corrected, 0 reject; sources 30 verified, 33 located, 0 missing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UXNR5K8zTWgEZFA3LQ7xCJ
</commit_message>
<xml_diff>
--- a/REVISION_CLINICA/revision_clinica.xlsx
+++ b/REVISION_CLINICA/revision_clinica.xlsx
@@ -5775,22 +5775,22 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Farmacología de agonistas beta-2 (relajan el útero); la hemorragia materna con inestabilidad contraindica los tocolíticos</t>
+          <t>Lee HL et al., Medicine 2020 (doi:10.1097/md.0000000000023651): los tocolíticos aumentan la hemorragia por atonía (betamiméticos aHR 1.71); FIGO 2022: oxitocina de primera línea</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Insufficient data: sin fuente específica localizada; el mecanismo (tocolítico) es farmacología básica</t>
+          <t>Solo la fuente: Lee 2020 (tocolíticos y hemorragia por atonía). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -5947,22 +5947,22 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>FIGO, recomendaciones de buena práctica en parto pretérmino; contraindicación absoluta de tocólisis en infección intraamniótica</t>
+          <t>CNGOF, Schmitz T et al., Eur J Obstet Gynecol Reprod Biol 2019 (doi:10.1016/j.ejogrb.2019.02.021): ante infección intrauterina, antibiótico IV inmediato y nacimiento temprano (grado A); ACOG Committee Opinion 712 (2017)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Insufficient data: fuente no localizada en PubMed</t>
+          <t>Solo la fuente: CNGOF 2019 (infección intrauterina: nacimiento temprano, grado A). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -6223,22 +6223,22 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>ACOG Practice Bulletin 222: Gestational Hypertension and Preeclampsia (2020)</t>
+          <t>Duley L et al., Magnesium sulphate versus diazepam for eclampsia, Cochrane 2010 (doi:10.1002/14651858.CD000127.pub2): menos muertes maternas (RR 0.59) y menos convulsiones recurrentes (RR 0.43); ACOG PB 222 (2020)</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>ACOG PB 222 no localizada en PubMed</t>
+          <t>Solo la fuente: Cochrane, Duley 2010. Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -8200,22 +8200,22 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>OMS/AIEPI, Plan C</t>
+          <t>OMS, Plan C; Houston KA et al., GASTRO, BMC Med 2019 (doi:10.1186/s12916-019-1356-z): Plan C = rehidratación IV con bolos para el choque; Maitland K et al., NEJM 2025 (doi:10.1056/NEJMoa2505752): bolos IV para el choque incluso en el brazo oral</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Plan C OMS/AIEPI no indexado</t>
+          <t>Solo la fuente: Houston 2019 y Maitland 2025 (choque = bolos IV). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -8528,22 +8528,22 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>OMS/AIEPI, Plan C</t>
+          <t>OMS, Plan C; Houston KA et al., GASTRO, BMC Med 2019 (doi:10.1186/s12916-019-1356-z): Plan C = rehidratación IV con bolos para el choque; Maitland K et al., NEJM 2025 (doi:10.1056/NEJMoa2505752): bolos IV para el choque incluso en el brazo oral</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Plan C OMS/AIEPI no indexado</t>
+          <t>Solo la fuente: Houston 2019 y Maitland 2025 (choque = bolos IV). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -9372,22 +9372,22 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>AAP, Clinical Report: Hypertrophic Pyloric Stenosis; Hernanz-Schulman, Radiology (2003)</t>
+          <t>Gilbertson LE et al., Anesth Analg 2019 (doi:10.1213/ane.0000000000004446): la alcalosis es una urgencia médica y se asocia a apnea; Spicer RD, Br J Surg 1982 (doi:10.1002/bjs.1800690304): corrección hidroelectrolítica preoperatoria esencial</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>La fuente citada ('AAP Clinical Report') no se localizó; Insufficient data</t>
+          <t>La fuente citada ('AAP Clinical Report') no existe en PubMed; sustituida por Gilbertson 2019 y Spicer 1982. Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -10383,22 +10383,22 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>APA, Practice Guideline for the Assessment and Treatment of Patients with Suicidal Behaviors (2010)</t>
+          <t>Mann JJ et al., JAMA 2005 (doi:10.1001/jama.294.16.2064) y Zalsman G et al., Lancet Psychiatry 2016 (doi:10.1016/s2215-0366(16)30030-x): restringir el acceso a medios letales, incluidos fármacos, previene el suicidio</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>APA 2010 no localizada en PubMed</t>
+          <t>Solo la fuente: Mann 2005, Zalsman 2016 (restricción de medios letales). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -10910,27 +10910,27 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Navarro: La clozapina exige vigilar el recuento de neutrófilos de forma periódica, porque puede causar agranulocitosis grave.</t>
+          <t>Navarro: La clozapina exige vigilar el recuento de neutrófilos de forma periódica, sobre todo en los primeros 2 años, porque puede causar agranulocitosis grave.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>APA, Practice Guideline for the Treatment of Patients with Schizophrenia (2020)</t>
+          <t>Siskind D et al., consenso Delphi global, Lancet Psychiatry 2025 (doi:10.1016/s2215-0366(25)00098-7): vigilancia de neutrófilos durante los primeros 2 años; Zhou H et al., Br J Psychiatry 2026: riesgo máximo en las primeras 18 semanas</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>APA 2020 no localizada en PubMed</t>
+          <t>Comentario: precisa los primeros 2 años (Siskind 2025, consenso Delphi global). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14314,22 +14314,22 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Farmacología de agonistas beta-2 (relajan el útero); la hemorragia materna con inestabilidad contraindica los tocolíticos</t>
+          <t>Lee HL et al., Medicine 2020 (doi:10.1097/md.0000000000023651): los tocolíticos aumentan la hemorragia por atonía (betamiméticos aHR 1.71); FIGO 2022: oxitocina de primera línea</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Insufficient data: sin fuente específica localizada; el mecanismo (tocolítico) es farmacología básica</t>
+          <t>Solo la fuente: Lee 2020 (tocolíticos y hemorragia por atonía). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14382,22 +14382,22 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>FIGO, recomendaciones de buena práctica en parto pretérmino; contraindicación absoluta de tocólisis en infección intraamniótica</t>
+          <t>CNGOF, Schmitz T et al., Eur J Obstet Gynecol Reprod Biol 2019 (doi:10.1016/j.ejogrb.2019.02.021): ante infección intrauterina, antibiótico IV inmediato y nacimiento temprano (grado A); ACOG Committee Opinion 712 (2017)</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Insufficient data: fuente no localizada en PubMed</t>
+          <t>Solo la fuente: CNGOF 2019 (infección intrauterina: nacimiento temprano, grado A). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14450,22 +14450,22 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>ACOG Practice Bulletin 222: Gestational Hypertension and Preeclampsia (2020)</t>
+          <t>Duley L et al., Magnesium sulphate versus diazepam for eclampsia, Cochrane 2010 (doi:10.1002/14651858.CD000127.pub2): menos muertes maternas (RR 0.59) y menos convulsiones recurrentes (RR 0.43); ACOG PB 222 (2020)</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>ACOG PB 222 no localizada en PubMed</t>
+          <t>Solo la fuente: Cochrane, Duley 2010. Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14586,22 +14586,22 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>OMS/AIEPI, Plan C</t>
+          <t>OMS, Plan C; Houston KA et al., GASTRO, BMC Med 2019 (doi:10.1186/s12916-019-1356-z): Plan C = rehidratación IV con bolos para el choque; Maitland K et al., NEJM 2025 (doi:10.1056/NEJMoa2505752): bolos IV para el choque incluso en el brazo oral</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Plan C OMS/AIEPI no indexado</t>
+          <t>Solo la fuente: Houston 2019 y Maitland 2025 (choque = bolos IV). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14654,22 +14654,22 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>OMS/AIEPI, Plan C</t>
+          <t>OMS, Plan C; Houston KA et al., GASTRO, BMC Med 2019 (doi:10.1186/s12916-019-1356-z): Plan C = rehidratación IV con bolos para el choque; Maitland K et al., NEJM 2025 (doi:10.1056/NEJMoa2505752): bolos IV para el choque incluso en el brazo oral</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Plan C OMS/AIEPI no indexado</t>
+          <t>Solo la fuente: Houston 2019 y Maitland 2025 (choque = bolos IV). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14926,22 +14926,22 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>AAP, Clinical Report: Hypertrophic Pyloric Stenosis; Hernanz-Schulman, Radiology (2003)</t>
+          <t>Gilbertson LE et al., Anesth Analg 2019 (doi:10.1213/ane.0000000000004446): la alcalosis es una urgencia médica y se asocia a apnea; Spicer RD, Br J Surg 1982 (doi:10.1002/bjs.1800690304): corrección hidroelectrolítica preoperatoria esencial</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>La fuente citada ('AAP Clinical Report') no se localizó; Insufficient data</t>
+          <t>La fuente citada ('AAP Clinical Report') no existe en PubMed; sustituida por Gilbertson 2019 y Spicer 1982. Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14994,22 +14994,22 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>APA, Practice Guideline for the Assessment and Treatment of Patients with Suicidal Behaviors (2010)</t>
+          <t>Mann JJ et al., JAMA 2005 (doi:10.1001/jama.294.16.2064) y Zalsman G et al., Lancet Psychiatry 2016 (doi:10.1016/s2215-0366(16)30030-x): restringir el acceso a medios letales, incluidos fármacos, previene el suicidio</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>APA 2010 no localizada en PubMed</t>
+          <t>Solo la fuente: Mann 2005, Zalsman 2016 (restricción de medios letales). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -15261,27 +15261,27 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>Navarro: La clozapina exige vigilar el recuento de neutrófilos de forma periódica, porque puede causar agranulocitosis grave.</t>
+          <t>Navarro: La clozapina exige vigilar el recuento de neutrófilos de forma periódica, sobre todo en los primeros 2 años, porque puede causar agranulocitosis grave.</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>APA, Practice Guideline for the Treatment of Patients with Schizophrenia (2020)</t>
+          <t>Siskind D et al., consenso Delphi global, Lancet Psychiatry 2025 (doi:10.1016/s2215-0366(25)00098-7): vigilancia de neutrófilos durante los primeros 2 años; Zhou H et al., Br J Psychiatry 2026: riesgo máximo en las primeras 18 semanas</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Aprobar</t>
+          <t>Corregir</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>APA 2020 no localizada en PubMed</t>
+          <t>Comentario: precisa los primeros 2 años (Siskind 2025, consenso Delphi global). Aplicada el 2026-10-13 (tools/apply_clinical_review_2026_10.py)</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>